<commit_message>
Use 178A CTF spec field names
</commit_message>
<xml_diff>
--- a/cases/c2m_8023dj_4p13p0_500mm/config/config_178A.xlsx
+++ b/cases/c2m_8023dj_4p13p0_500mm/config/config_178A.xlsx
@@ -928,7 +928,7 @@
       </c>
       <c r="B20" s="15" t="inlineStr">
         <is>
-          <t>f_z</t>
+          <t>f_z1</t>
         </is>
       </c>
       <c r="C20" s="16" t="n">
@@ -941,7 +941,7 @@
       </c>
       <c r="E20" s="15" t="inlineStr">
         <is>
-          <t>178A/93A aligned main CTF zero; sourced from COM Ad Hoc f_z.</t>
+          <t>178A CTF zero 1; sourced from COM Ad Hoc f_z.</t>
         </is>
       </c>
     </row>
@@ -953,7 +953,7 @@
       </c>
       <c r="B21" s="15" t="inlineStr">
         <is>
-          <t>f_LF</t>
+          <t>f_z2</t>
         </is>
       </c>
       <c r="C21" s="16" t="n">
@@ -966,7 +966,7 @@
       </c>
       <c r="E21" s="15" t="inlineStr">
         <is>
-          <t>178A/93A aligned low-frequency pole/zero; sourced from COM Ad Hoc f_HP_PZ.</t>
+          <t>178A CTF zero 2; aligned 93A COM Ad Hoc f_HP_PZ mapping.</t>
         </is>
       </c>
     </row>
@@ -1031,7 +1031,9 @@
           <t>f_p3</t>
         </is>
       </c>
-      <c r="C24" s="16" t="n"/>
+      <c r="C24" s="16" t="n">
+        <v>1328125000</v>
+      </c>
       <c r="D24" s="15" t="inlineStr">
         <is>
           <t>Hz</t>
@@ -1039,7 +1041,7 @@
       </c>
       <c r="E24" s="15" t="inlineStr">
         <is>
-          <t>Optional 178A CTF pole 3; leave blank to bypass the third pole.</t>
+          <t>178A CTF pole 3; aligned 93A COM Ad Hoc f_HP_PZ mapping.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix project channel enable parsing
</commit_message>
<xml_diff>
--- a/cases/c2m_8023dj_4p13p0_500mm/config/config_178A.xlsx
+++ b/cases/c2m_8023dj_4p13p0_500mm/config/config_178A.xlsx
@@ -486,7 +486,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="12">
       <c r="A3" s="14" t="inlineStr">
         <is>
@@ -4325,9 +4324,8 @@
       <c r="G4" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H4" s="15">
-        <f>TRUE()</f>
-        <v/>
+      <c r="H4" s="15" t="b">
+        <v>1</v>
       </c>
       <c r="I4" s="15" t="inlineStr">
         <is>
@@ -4363,9 +4361,8 @@
       <c r="G5" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H5" s="15">
-        <f>TRUE()</f>
-        <v/>
+      <c r="H5" s="15" t="b">
+        <v>1</v>
       </c>
       <c r="I5" s="15" t="inlineStr">
         <is>
@@ -4401,9 +4398,8 @@
       <c r="G6" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H6" s="15">
-        <f>TRUE()</f>
-        <v/>
+      <c r="H6" s="15" t="b">
+        <v>1</v>
       </c>
       <c r="I6" s="15" t="inlineStr">
         <is>
@@ -4439,9 +4435,8 @@
       <c r="G7" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H7" s="15">
-        <f>TRUE()</f>
-        <v/>
+      <c r="H7" s="15" t="b">
+        <v>1</v>
       </c>
       <c r="I7" s="15" t="inlineStr">
         <is>
@@ -4477,9 +4472,8 @@
       <c r="G8" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H8" s="15">
-        <f>TRUE()</f>
-        <v/>
+      <c r="H8" s="15" t="b">
+        <v>1</v>
       </c>
       <c r="I8" s="15" t="inlineStr">
         <is>
@@ -4515,9 +4509,8 @@
       <c r="G9" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H9" s="15">
-        <f>TRUE()</f>
-        <v/>
+      <c r="H9" s="15" t="b">
+        <v>1</v>
       </c>
       <c r="I9" s="15" t="inlineStr">
         <is>
@@ -4553,9 +4546,8 @@
       <c r="G10" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H10" s="15">
-        <f>TRUE()</f>
-        <v/>
+      <c r="H10" s="15" t="b">
+        <v>1</v>
       </c>
       <c r="I10" s="15" t="inlineStr">
         <is>
@@ -4591,9 +4583,8 @@
       <c r="G11" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H11" s="15">
-        <f>TRUE()</f>
-        <v/>
+      <c r="H11" s="15" t="b">
+        <v>1</v>
       </c>
       <c r="I11" s="15" t="inlineStr">
         <is>
@@ -4629,9 +4620,8 @@
       <c r="G12" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H12" s="15">
-        <f>TRUE()</f>
-        <v/>
+      <c r="H12" s="15" t="b">
+        <v>1</v>
       </c>
       <c r="I12" s="15" t="inlineStr">
         <is>
@@ -4667,9 +4657,8 @@
       <c r="G13" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H13" s="15">
-        <f>TRUE()</f>
-        <v/>
+      <c r="H13" s="15" t="b">
+        <v>1</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -4705,9 +4694,8 @@
       <c r="G14" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H14" s="15">
-        <f>TRUE()</f>
-        <v/>
+      <c r="H14" s="15" t="b">
+        <v>1</v>
       </c>
       <c r="I14" s="15" t="inlineStr">
         <is>
@@ -4743,9 +4731,8 @@
       <c r="G15" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="H15" s="15">
-        <f>TRUE()</f>
-        <v/>
+      <c r="H15" s="15" t="b">
+        <v>1</v>
       </c>
       <c r="I15" s="15" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Enable 178A full search dimensions
</commit_message>
<xml_diff>
--- a/cases/c2m_8023dj_4p13p0_500mm/config/config_178A.xlsx
+++ b/cases/c2m_8023dj_4p13p0_500mm/config/config_178A.xlsx
@@ -4017,9 +4017,8 @@
           <t>c_m2</t>
         </is>
       </c>
-      <c r="B4" s="15">
-        <f>TRUE()</f>
-        <v/>
+      <c r="B4" s="15" t="b">
+        <v>1</v>
       </c>
       <c r="C4" s="16" t="inlineStr">
         <is>
@@ -4043,9 +4042,8 @@
           <t>c_m1</t>
         </is>
       </c>
-      <c r="B5" s="15">
-        <f>TRUE()</f>
-        <v/>
+      <c r="B5" s="15" t="b">
+        <v>1</v>
       </c>
       <c r="C5" s="16" t="inlineStr">
         <is>
@@ -4069,9 +4067,8 @@
           <t>c_1</t>
         </is>
       </c>
-      <c r="B6" s="15">
-        <f>TRUE()</f>
-        <v/>
+      <c r="B6" s="15" t="b">
+        <v>1</v>
       </c>
       <c r="C6" s="16" t="inlineStr">
         <is>
@@ -4095,9 +4092,8 @@
           <t>g_1</t>
         </is>
       </c>
-      <c r="B7" s="15">
-        <f>TRUE()</f>
-        <v/>
+      <c r="B7" s="15" t="b">
+        <v>1</v>
       </c>
       <c r="C7" s="16" t="inlineStr">
         <is>
@@ -4121,9 +4117,8 @@
           <t>g_2</t>
         </is>
       </c>
-      <c r="B8" s="15">
-        <f>TRUE()</f>
-        <v/>
+      <c r="B8" s="15" t="b">
+        <v>1</v>
       </c>
       <c r="C8" s="16" t="inlineStr">
         <is>

</xml_diff>